<commit_message>
programming workstation - add and create and program and instructions
</commit_message>
<xml_diff>
--- a/devices/TR/IP_TEMPLATE.xlsx
+++ b/devices/TR/IP_TEMPLATE.xlsx
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -173,6 +173,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1166,7 +1169,7 @@
         </is>
       </c>
       <c r="H3" s="17" t="n">
-        <v>46191.36578709491</v>
+        <v>46196.45684946759</v>
       </c>
       <c r="I3" s="10" t="inlineStr">
         <is>
@@ -1184,7 +1187,7 @@
         </is>
       </c>
       <c r="L3" s="21" t="n">
-        <v>46191.36625766632</v>
+        <v>46196.45684671296</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -1192,7 +1195,7 @@
         </is>
       </c>
       <c r="N3" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -1226,7 +1229,7 @@
         </is>
       </c>
       <c r="H4" s="17" t="n">
-        <v>46191.32725549769</v>
+        <v>46196.52679668982</v>
       </c>
       <c r="I4" s="18" t="inlineStr">
         <is>
@@ -1244,15 +1247,15 @@
         </is>
       </c>
       <c r="L4" s="24" t="n">
-        <v>46191.32772528935</v>
-      </c>
-      <c r="M4" s="1" t="inlineStr">
+        <v>46196.52679421296</v>
+      </c>
+      <c r="M4" s="18" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
       <c r="N4" s="22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -1556,8 +1559,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>